<commit_message>
docs: reconcile system test evidence
</commit_message>
<xml_diff>
--- a/tests/FocusMate_Test/Excel/FocusMate_24_Test_Cases_Severity.xlsx
+++ b/tests/FocusMate_Test/Excel/FocusMate_24_Test_Cases_Severity.xlsx
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="334" uniqueCount="222">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="248" uniqueCount="248">
   <si>
     <t>ID</t>
   </si>
@@ -703,6 +703,84 @@
   </si>
   <si>
     <t>TC22_Reconnect</t>
+  </si>
+  <si>
+    <t>TC03_camera.png</t>
+  </si>
+  <si>
+    <t>TC04_web.png</t>
+  </si>
+  <si>
+    <t>TC05_camera_web.png</t>
+  </si>
+  <si>
+    <t>TC06_session_start.jpg</t>
+  </si>
+  <si>
+    <t>TC07_normal_pose_web.png</t>
+  </si>
+  <si>
+    <t>TC08_head_down.png</t>
+  </si>
+  <si>
+    <t>TC09_tilt_left.png</t>
+  </si>
+  <si>
+    <t>TC10_tilt_right.png</t>
+  </si>
+  <si>
+    <t>TC11_slouch.png</t>
+  </si>
+  <si>
+    <t>TC12_yawn.png</t>
+  </si>
+  <si>
+    <t>TC_13.mp4</t>
+  </si>
+  <si>
+    <t>TC14_ai_repeated.png</t>
+  </si>
+  <si>
+    <t>test_canhbao.mp4</t>
+  </si>
+  <si>
+    <t>Test_rungnhe_canhbao_ngap.mp4</t>
+  </si>
+  <si>
+    <t>thongke_w.jpg; thongke_watch.jpg</t>
+  </si>
+  <si>
+    <t>TC19_session_events.jpg; TC19_summary_suggestion.jpg</t>
+  </si>
+  <si>
+    <t>TC20_session_end.jpg; test_khi-ketthuc.mp4</t>
+  </si>
+  <si>
+    <t>TC21_Dis.mp4</t>
+  </si>
+  <si>
+    <t>TC22_Reconnect.mp4</t>
+  </si>
+  <si>
+    <t>test_demo_web.mp4; test_canhbao.mp4; test_khi-ketthuc.mp4</t>
+  </si>
+  <si>
+    <t>TC24_Phiendai.jpg; TC24_Start_ss.png; TC24_KetThucPhienDongHo.mp4</t>
+  </si>
+  <si>
+    <t>Cố tình ngồi gần</t>
+  </si>
+  <si>
+    <t>Chạy liên tục khoảng 61 phút</t>
+  </si>
+  <si>
+    <t>Không crash/reset/mất dữ liệu bất thường trong suốt 61 phút</t>
+  </si>
+  <si>
+    <t>Chạy phiên 61 phút; hệ thống không crash/reset và tạo báo cáo</t>
+  </si>
+  <si>
+    <t>Phiên thực tế 61 phút; bắt đầu và kết thúc được ghi nhận</t>
   </si>
 </sst>
 </file>
@@ -1104,9 +1182,9 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:ns3="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:ns4="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ns1:Ignorable="x14ac xr xr2 xr3" ns2:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:M25"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15" ns3:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10" style="6" customWidth="1"/>
     <col min="2" max="2" width="16" style="6" customWidth="1"/>
@@ -1124,7 +1202,7 @@
     <col min="14" max="16384" width="9.140625" style="6"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:13" ns3:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1165,7 +1243,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="2" spans="1:13" ht="54.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:13" ht="54.95" customHeight="1" ns3:dyDescent="0.25">
       <c r="A2" s="7" t="s">
         <v>13</v>
       </c>
@@ -1206,7 +1284,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="3" spans="1:13" ht="54.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:13" ht="54.95" customHeight="1" ns3:dyDescent="0.25">
       <c r="A3" s="7" t="s">
         <v>20</v>
       </c>
@@ -1247,7 +1325,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="4" spans="1:13" ht="54.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:13" ht="54.95" customHeight="1" ns3:dyDescent="0.25">
       <c r="A4" s="7" t="s">
         <v>27</v>
       </c>
@@ -1276,7 +1354,7 @@
         <v>147</v>
       </c>
       <c r="J4" s="6" t="s">
-        <v>155</v>
+        <v>222</v>
       </c>
       <c r="K4" s="8" t="s">
         <v>149</v>
@@ -1288,7 +1366,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="5" spans="1:13" ht="54.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:13" ht="54.95" customHeight="1" ns3:dyDescent="0.25">
       <c r="A5" s="7" t="s">
         <v>33</v>
       </c>
@@ -1317,7 +1395,7 @@
         <v>147</v>
       </c>
       <c r="J5" s="6" t="s">
-        <v>159</v>
+        <v>223</v>
       </c>
       <c r="K5" s="8" t="s">
         <v>149</v>
@@ -1329,7 +1407,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="6" spans="1:13" ht="54.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:13" ht="54.95" customHeight="1" ns3:dyDescent="0.25">
       <c r="A6" s="7" t="s">
         <v>39</v>
       </c>
@@ -1358,7 +1436,7 @@
         <v>147</v>
       </c>
       <c r="J6" s="7" t="s">
-        <v>161</v>
+        <v>224</v>
       </c>
       <c r="K6" s="8" t="s">
         <v>217</v>
@@ -1370,7 +1448,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="7" spans="1:13" ht="54.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:13" ht="54.95" customHeight="1" ns3:dyDescent="0.25">
       <c r="A7" s="7" t="s">
         <v>46</v>
       </c>
@@ -1399,7 +1477,7 @@
         <v>147</v>
       </c>
       <c r="J7" s="6" t="s">
-        <v>164</v>
+        <v>225</v>
       </c>
       <c r="K7" s="8" t="s">
         <v>149</v>
@@ -1411,7 +1489,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="8" spans="1:13" ht="54.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:13" ht="54.95" customHeight="1" ns3:dyDescent="0.25">
       <c r="A8" s="7" t="s">
         <v>52</v>
       </c>
@@ -1440,7 +1518,7 @@
         <v>147</v>
       </c>
       <c r="J8" s="6" t="s">
-        <v>168</v>
+        <v>226</v>
       </c>
       <c r="K8" s="8" t="s">
         <v>149</v>
@@ -1452,7 +1530,7 @@
         <v>169</v>
       </c>
     </row>
-    <row r="9" spans="1:13" ht="54.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:13" ht="54.95" customHeight="1" ns3:dyDescent="0.25">
       <c r="A9" s="7" t="s">
         <v>58</v>
       </c>
@@ -1481,7 +1559,7 @@
         <v>147</v>
       </c>
       <c r="J9" s="6" t="s">
-        <v>171</v>
+        <v>227</v>
       </c>
       <c r="K9" s="8" t="s">
         <v>149</v>
@@ -1493,7 +1571,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="10" spans="1:13" ht="54.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:13" ht="54.95" customHeight="1" ns3:dyDescent="0.25">
       <c r="A10" s="7" t="s">
         <v>63</v>
       </c>
@@ -1522,7 +1600,7 @@
         <v>147</v>
       </c>
       <c r="J10" s="6" t="s">
-        <v>173</v>
+        <v>228</v>
       </c>
       <c r="K10" s="8" t="s">
         <v>149</v>
@@ -1534,7 +1612,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="11" spans="1:13" ht="54.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:13" ht="54.95" customHeight="1" ns3:dyDescent="0.25">
       <c r="A11" s="7" t="s">
         <v>67</v>
       </c>
@@ -1563,7 +1641,7 @@
         <v>147</v>
       </c>
       <c r="J11" s="6" t="s">
-        <v>175</v>
+        <v>229</v>
       </c>
       <c r="K11" s="8" t="s">
         <v>149</v>
@@ -1575,7 +1653,7 @@
         <v>209</v>
       </c>
     </row>
-    <row r="12" spans="1:13" ht="54.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:13" ht="54.95" customHeight="1" ns3:dyDescent="0.25">
       <c r="A12" s="7" t="s">
         <v>71</v>
       </c>
@@ -1592,7 +1670,7 @@
         <v>72</v>
       </c>
       <c r="F12" s="7" t="s">
-        <v>205</v>
+        <v>243</v>
       </c>
       <c r="G12" s="7" t="s">
         <v>206</v>
@@ -1604,7 +1682,7 @@
         <v>147</v>
       </c>
       <c r="J12" s="6" t="s">
-        <v>176</v>
+        <v>230</v>
       </c>
       <c r="K12" s="8" t="s">
         <v>149</v>
@@ -1616,7 +1694,7 @@
         <v>208</v>
       </c>
     </row>
-    <row r="13" spans="1:13" ht="54.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:13" ht="54.95" customHeight="1" ns3:dyDescent="0.25">
       <c r="A13" s="7" t="s">
         <v>73</v>
       </c>
@@ -1645,7 +1723,7 @@
         <v>147</v>
       </c>
       <c r="J13" s="6" t="s">
-        <v>178</v>
+        <v>231</v>
       </c>
       <c r="K13" s="8" t="s">
         <v>149</v>
@@ -1657,7 +1735,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="14" spans="1:13" ht="54.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:13" ht="54.95" customHeight="1" ns3:dyDescent="0.25">
       <c r="A14" s="7" t="s">
         <v>77</v>
       </c>
@@ -1686,7 +1764,7 @@
         <v>147</v>
       </c>
       <c r="J14" s="6" t="s">
-        <v>181</v>
+        <v>232</v>
       </c>
       <c r="K14" s="8" t="s">
         <v>149</v>
@@ -1698,7 +1776,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="15" spans="1:13" ht="54.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:13" ht="54.95" customHeight="1" ns3:dyDescent="0.25">
       <c r="A15" s="7" t="s">
         <v>80</v>
       </c>
@@ -1727,7 +1805,7 @@
         <v>147</v>
       </c>
       <c r="J15" s="6" t="s">
-        <v>184</v>
+        <v>233</v>
       </c>
       <c r="K15" s="8" t="s">
         <v>149</v>
@@ -1739,7 +1817,7 @@
         <v>185</v>
       </c>
     </row>
-    <row r="16" spans="1:13" ht="54.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:13" ht="54.95" customHeight="1" ns3:dyDescent="0.25">
       <c r="A16" s="7" t="s">
         <v>84</v>
       </c>
@@ -1768,7 +1846,7 @@
         <v>147</v>
       </c>
       <c r="J16" s="6" t="s">
-        <v>213</v>
+        <v>234</v>
       </c>
       <c r="K16" s="8" t="s">
         <v>149</v>
@@ -1780,7 +1858,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="17" spans="1:13" ht="54.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:13" ht="54.95" customHeight="1" ns3:dyDescent="0.25">
       <c r="A17" s="7" t="s">
         <v>90</v>
       </c>
@@ -1809,7 +1887,7 @@
         <v>147</v>
       </c>
       <c r="J17" s="6" t="s">
-        <v>213</v>
+        <v>234</v>
       </c>
       <c r="K17" s="8" t="s">
         <v>149</v>
@@ -1821,7 +1899,7 @@
         <v>189</v>
       </c>
     </row>
-    <row r="18" spans="1:13" ht="54.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:13" ht="54.95" customHeight="1" ns3:dyDescent="0.25">
       <c r="A18" s="7" t="s">
         <v>96</v>
       </c>
@@ -1850,7 +1928,7 @@
         <v>147</v>
       </c>
       <c r="J18" s="6" t="s">
-        <v>213</v>
+        <v>235</v>
       </c>
       <c r="K18" s="8" t="s">
         <v>149</v>
@@ -1862,7 +1940,7 @@
         <v>191</v>
       </c>
     </row>
-    <row r="19" spans="1:13" ht="54.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:13" ht="54.95" customHeight="1" ns3:dyDescent="0.25">
       <c r="A19" s="7" t="s">
         <v>99</v>
       </c>
@@ -1891,7 +1969,7 @@
         <v>147</v>
       </c>
       <c r="J19" s="6" t="s">
-        <v>194</v>
+        <v>236</v>
       </c>
       <c r="K19" s="8" t="s">
         <v>149</v>
@@ -1903,7 +1981,7 @@
         <v>193</v>
       </c>
     </row>
-    <row r="20" spans="1:13" ht="54.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:13" ht="54.95" customHeight="1" ns3:dyDescent="0.25">
       <c r="A20" s="7" t="s">
         <v>105</v>
       </c>
@@ -1932,7 +2010,7 @@
         <v>147</v>
       </c>
       <c r="J20" s="6" t="s">
-        <v>203</v>
+        <v>237</v>
       </c>
       <c r="K20" s="8" t="s">
         <v>149</v>
@@ -1944,7 +2022,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="21" spans="1:13" ht="54.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:13" ht="54.95" customHeight="1" ns3:dyDescent="0.25">
       <c r="A21" s="7" t="s">
         <v>110</v>
       </c>
@@ -1981,8 +2059,11 @@
       <c r="M21" s="6" t="s">
         <v>197</v>
       </c>
-    </row>
-    <row r="22" spans="1:13" ht="54.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="J21" t="s" s="6">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="22" spans="1:13" ht="54.95" customHeight="1" ns3:dyDescent="0.25">
       <c r="A22" s="7" t="s">
         <v>114</v>
       </c>
@@ -2011,7 +2092,7 @@
         <v>147</v>
       </c>
       <c r="J22" s="6" t="s">
-        <v>220</v>
+        <v>239</v>
       </c>
       <c r="K22" s="8" t="s">
         <v>217</v>
@@ -2023,7 +2104,7 @@
         <v>199</v>
       </c>
     </row>
-    <row r="23" spans="1:13" ht="54.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:13" ht="54.95" customHeight="1" ns3:dyDescent="0.25">
       <c r="A23" s="7" t="s">
         <v>120</v>
       </c>
@@ -2052,7 +2133,7 @@
         <v>147</v>
       </c>
       <c r="J23" s="6" t="s">
-        <v>221</v>
+        <v>240</v>
       </c>
       <c r="K23" s="8" t="s">
         <v>217</v>
@@ -2064,7 +2145,7 @@
         <v>201</v>
       </c>
     </row>
-    <row r="24" spans="1:13" ht="54.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:13" ht="54.95" customHeight="1" ns3:dyDescent="0.25">
       <c r="A24" s="7" t="s">
         <v>125</v>
       </c>
@@ -2093,7 +2174,7 @@
         <v>147</v>
       </c>
       <c r="J24" s="7" t="s">
-        <v>214</v>
+        <v>241</v>
       </c>
       <c r="K24" s="8" t="s">
         <v>217</v>
@@ -2103,7 +2184,7 @@
       </c>
       <c r="M24" s="7"/>
     </row>
-    <row r="25" spans="1:13" ht="54.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:13" ht="54.95" customHeight="1" ns3:dyDescent="0.25">
       <c r="A25" s="7" t="s">
         <v>131</v>
       </c>
@@ -2120,19 +2201,19 @@
         <v>128</v>
       </c>
       <c r="F25" s="7" t="s">
-        <v>218</v>
+        <v>244</v>
       </c>
       <c r="G25" s="7" t="s">
-        <v>134</v>
+        <v>245</v>
       </c>
       <c r="H25" s="7" t="s">
-        <v>219</v>
+        <v>246</v>
       </c>
       <c r="I25" s="7" t="s">
         <v>147</v>
       </c>
       <c r="J25" s="7" t="s">
-        <v>215</v>
+        <v>242</v>
       </c>
       <c r="K25" s="8" t="s">
         <v>217</v>
@@ -2141,22 +2222,22 @@
         <v>150</v>
       </c>
       <c r="M25" s="7" t="s">
-        <v>216</v>
+        <v>247</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:M25" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
+  <autoFilter ref="A1:M25" ns2:uid="{00000000-0009-0000-0000-000000000000}"/>
   <phoneticPr fontId="4" type="noConversion"/>
   <dataValidations count="2">
-    <dataValidation type="list" errorTitle="Severity không hợp lệ" error="Chọn Critical, High, Medium hoặc Low." sqref="D2:D25" xr:uid="{00000000-0002-0000-0000-000000000000}">
+    <dataValidation type="list" errorTitle="Severity không hợp lệ" error="Chọn Critical, High, Medium hoặc Low." sqref="D2:D25" ns2:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"Critical,High,Medium,Low"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" errorTitle="Kết quả không hợp lệ" error="Chọn PASS hoặc FAIL." sqref="I2:I25" xr:uid="{00000000-0002-0000-0000-000001000000}">
+    <dataValidation type="list" allowBlank="1" errorTitle="Kết quả không hợp lệ" error="Chọn PASS hoặc FAIL." sqref="I2:I25" ns2:uid="{00000000-0002-0000-0000-000001000000}">
       <formula1>"PASS,FAIL"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup orientation="portrait" r:id="rId1"/>
+  <pageSetup orientation="portrait" ns4:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>